<commit_message>
Attribute product costs by style_family instead of per-SKU
Small teams find per-SKU cost tagging hard, so COSTS now attributes production
spend at the style-family level:
- COSTS: sku column -> style_family (links to INVENTORY.style_family).
- Dashboard 'Where money went': new 'Product cost by style family' card —
  spend per family with a rough make-cost per piece (family spend / pieces),
  plus updated sheet-hygiene tip.
- Data mapping reads style_family (falls back to sku); inventory exposes
  style_family for the join.
- Updated workbook (COSTS style_family + family dropdown, refreshed How-to)
  and data-model doc.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -951,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -977,7 +977,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>THE KEY IDEA — SKU ties every tab together</t>
+          <t>THE KEY IDEA — SKU ties the tabs together</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>INVENTORY.sku (the piece) = REVENUE.sku (what sold) = COSTS.sku (what it cost to make). style_family keeps your grouping code.</t>
+          <t>INVENTORY.sku = the piece · REVENUE.sku = what sold · style_family groups pieces.</t>
         </is>
       </c>
     </row>
@@ -1015,91 +1015,63 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>INVENTORY — one row per finished piece; unique sku; unit_cost = make cost (lower), unit_price = selling price (higher).</t>
+          <t>INVENTORY — one row per finished piece; unique sku; style_family = your grouping code; unit_cost = make cost (lower), unit_price = selling price (higher).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>REVENUE — one row per sale; put the exact piece sku; fill revenue (the sale amount) and units_sold.</t>
+          <t>REVENUE — one row per sale; exact piece sku; fill revenue (the sale amount) and units_sold.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>COSTS — one row per expense; cost_function = Product / Marketing &amp; brand / Overheads; tag sku for production spend to get true per-piece cost.</t>
+          <t>COSTS — one row per expense; cost_function = Product / Marketing &amp; brand / Overheads. For production spend put the style_family (e.g. HB1HE) — costs roll up per family (lighter than per-SKU while small).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>CHANNELS — one row per date × channel (impressions, clicks, conversions, cost). channel_name must match REVENUE.channel.</t>
+          <t>CHANNELS — one row per date × channel.  CUSTOMERS — one row per customer.  ALERTS — the action board.  TARGETS — monthly plan.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>CUSTOMERS — one row per customer (age_band, gender power the audience; LTV &amp; repeat are derived).</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>ALERTS — the app's action board reads &amp; writes this.  TARGETS — monthly plan for 'vs target'.</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATERIALS — raw-material stock at a glance</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>No exact meters needed. Set status = In stock / Running low / Out of stock, and on_order = Yes when it's on the way. quantity_on_hand &amp; reorder_level are optional.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>MATERIALS (new) — raw-material stock at a glance</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>You don't need exact meters. Set status = In stock / Running low / Out of stock, and on_order = Yes when it's on the way. quantity_on_hand &amp; reorder_level are optional estimates.</t>
+          <t>SKU_MATERIALS (optional) — link a material to the pieces that use it: sku, material, qty_used, unit, notes.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Columns: material, category (Fabric/Thread/Paint/Button/Trim/Packaging/Article/Other), unit, quantity_on_hand, reorder_level, status, on_order, expected_date, supplier, notes.</t>
-        </is>
-      </c>
+      <c r="A19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>SKU_MATERIALS (optional) — link materials to pieces</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Only if you want to know which pieces use a material (e.g. 'this fabric goes into these SKUs'). One row per sku × material: sku, material, qty_used, unit, notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
         </is>
@@ -3844,7 +3816,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
@@ -3907,7 +3879,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>sku</t>
+          <t>style_family</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -5054,6 +5026,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reflect style_family across tabs (REVENUE + Sales + Costs)
- REVENUE now carries both sku (exact piece) and style_family (the group);
  the mapping derives style_family from the sku prefix when left blank.
- Sales & channels: new 'Revenue by style family' card, mirroring the
  cost-by-family view on Where money went.
- Where money went: family card upgraded to 'Style family economics' —
  make-cost, revenue, net and category mix per family (jacket & accessory
  stay separate via category, never merged by family).
- Workbook: REVENUE gains a style_family column (+ family-code dropdown);
  refreshed How-to. Data-model doc updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -476,27 +476,6 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,27 +504,6 @@
           <t>gst_registered</t>
         </is>
       </c>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -589,27 +547,6 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -638,27 +575,6 @@
           <t>due_date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -951,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -977,21 +893,21 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>THE KEY IDEA — SKU ties the tabs together</t>
+          <t>THE KEY IDEA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>A SKU is like a barcode on ONE physical piece — unique, never shared. Your family code (brand+collection+technique, e.g. HB1HE) is a PREFIX; add a number per piece: HB1HE-01, HB1HE-02…</t>
+          <t>sku = one physical piece (unique, e.g. HB1HE-01).  style_family = the group (brand+collection+technique, e.g. HB1HE).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>INVENTORY.sku = the piece · REVENUE.sku = what sold · style_family groups pieces.</t>
+          <t>Both appear on INVENTORY, REVENUE and COSTS so everything links: a sale points to the exact piece (sku) AND rolls up to the family (style_family).</t>
         </is>
       </c>
     </row>
@@ -1008,70 +924,60 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>MASTER — one config row.  BRANDS — one row per brand.</t>
+          <t>INVENTORY — one row per finished piece; unique sku + style_family; unit_cost = make cost (lower), unit_price = selling price (higher).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>INVENTORY — one row per finished piece; unique sku; style_family = your grouping code; unit_cost = make cost (lower), unit_price = selling price (higher).</t>
+          <t>REVENUE — one row per sale; put both sku (exact piece) and style_family; fill revenue and units_sold.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>REVENUE — one row per sale; exact piece sku; fill revenue (the sale amount) and units_sold.</t>
+          <t>COSTS — one row per expense; cost_function; for production spend put style_family so costs roll up per family.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>COSTS — one row per expense; cost_function = Product / Marketing &amp; brand / Overheads. For production spend put the style_family (e.g. HB1HE) — costs roll up per family (lighter than per-SKU while small).</t>
+          <t>CHANNELS · CUSTOMERS · ALERTS · TARGETS — as before.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>CHANNELS — one row per date × channel.  CUSTOMERS — one row per customer.  ALERTS — the action board.  TARGETS — monthly plan.</t>
-        </is>
-      </c>
+      <c r="A13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>MATERIALS — raw stock at a glance: status (In stock / Running low / Out of stock) + on_order. Quantities optional.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>MATERIALS — raw-material stock at a glance</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>SKU_MATERIALS (optional) — link a material to the pieces that use it.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>No exact meters needed. Set status = In stock / Running low / Out of stock, and on_order = Yes when it's on the way. quantity_on_hand &amp; reorder_level are optional.</t>
-        </is>
-      </c>
+      <c r="A16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Jacket and accessory always stay separate — breakdowns use category/silhouette, never merged by family.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>SKU_MATERIALS (optional) — link a material to the pieces that use it: sku, material, qty_used, unit, notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
         </is>
@@ -1095,28 +1001,6 @@
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1140,28 +1024,6 @@
           <t>status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3463,35 +3325,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3512,71 +3363,64 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>style_family</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>collection</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>revenue</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>units_sold</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>discount_amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>returns_units</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>returns_value</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Product_name</t>
         </is>
       </c>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3596,41 +3440,46 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>HB1PHE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>8000</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>4000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Compliments</t>
         </is>
@@ -3654,41 +3503,46 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>HB1HE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>10000</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>100</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>2</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Harm the harmonium</t>
         </is>
@@ -3712,26 +3566,31 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>HB1UHE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Handkerchief</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Black with face in the centre</t>
         </is>
@@ -3755,46 +3614,58 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>HB1UHE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Retail</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Handkerchief</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="E16" t="inlineStr">
+    <row r="6">
+      <c r="D6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
         <is>
           <t xml:space="preserve">Integrate product name </t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="E17" t="inlineStr">
+    <row r="7">
+      <c r="D7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
         <is>
           <t>Integrate unit price</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3819,21 +3690,6 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3892,21 +3748,6 @@
           <t>paid</t>
         </is>
       </c>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5050,26 +4891,6 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5103,26 +4924,6 @@
           <t>cost</t>
         </is>
       </c>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5182,24 +4983,6 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5243,24 +5026,6 @@
           <t>acquisition_cost</t>
         </is>
       </c>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
-      <c r="Z1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
Add size as a piece-level attribute (INVENTORY + REVENUE)
Size drives per-piece cost, so it lives at the piece level: each size is its
own INVENTORY row with its own unit_cost. Adds:
- INVENTORY.size and REVENUE.size columns (dropdown XS…XXL / Free Size / Custom).
- Data mapping reads size on inventory and revenue.
- Inventory screen: 'Units by size' breakdown + size shown per piece in the
  stock ledger (e.g. 'Shirt · M').
- Workbook + data-model doc updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -867,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -907,77 +907,84 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Both appear on INVENTORY, REVENUE and COSTS so everything links: a sale points to the exact piece (sku) AND rolls up to the family (style_family).</t>
+          <t>Size is a piece-level attribute: each size is its own INVENTORY row with its own unit_cost, so an L that costs more than an M is captured automatically.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Both sku and style_family appear on INVENTORY, REVENUE and COSTS so everything links.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>TABS</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>INVENTORY — one row per finished piece; unique sku + style_family; unit_cost = make cost (lower), unit_price = selling price (higher).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>REVENUE — one row per sale; put both sku (exact piece) and style_family; fill revenue and units_sold.</t>
+          <t>INVENTORY — one row per finished piece; unique sku + style_family; size (XS…XXL/Free Size/Custom); unit_cost = make cost, unit_price = selling price.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>COSTS — one row per expense; cost_function; for production spend put style_family so costs roll up per family.</t>
+          <t>REVENUE — one row per sale; sku + style_family + size sold; revenue and units_sold.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>COSTS — one row per expense; cost_function; production spend gets a style_family so costs roll up per family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>CHANNELS · CUSTOMERS · ALERTS · TARGETS — as before.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>MATERIALS — raw stock at a glance: status (In stock / Running low / Out of stock) + on_order. Quantities optional.</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>MATERIALS — raw stock at a glance: status (In stock / Running low / Out of stock) + on_order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>SKU_MATERIALS (optional) — link a material to the pieces that use it.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Jacket and accessory always stay separate — breakdowns use category/silhouette, never merged by family.</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Jacket and accessory always stay separate — breakdowns use category/silhouette, never merged by family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
         </is>
@@ -1080,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1088,18 +1095,19 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1130,60 +1138,65 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>collection</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fabric</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>unit_cost</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>unit_price</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>quantity_on_hand</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>reorder_level</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>warehouse</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>silhouette</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>proportion</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>technique</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>colour</t>
         </is>
@@ -1215,51 +1228,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Bamboo</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>2200</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>9595</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t xml:space="preserve">Short Sleeve Shirt + Running Embroidery </t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Digital print + Hand Embroidery</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Indigo Blue</t>
         </is>
@@ -1291,51 +1304,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>100% Linen</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>2500</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>8585</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t xml:space="preserve">Long Sleeve Shirt  + Small Object Hand Embroidery  </t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Olive Green</t>
         </is>
@@ -1367,51 +1380,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed: Cotton + Linen </t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>2600</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>9999</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t xml:space="preserve">Short Sleeve + Long Crop Top + Medium Embroidery </t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t xml:space="preserve">White </t>
         </is>
@@ -1443,51 +1456,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Mixed: Cotton + Linen</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>2800</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>10100</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Short Sleeve Shirt + Hand Embroidery on Neck</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t xml:space="preserve">Off-White </t>
         </is>
@@ -1519,51 +1532,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Bamboo</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>3000</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>12345</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>1</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t xml:space="preserve">Short Crop Shirt + Full Hand Embroidery  </t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t xml:space="preserve">White </t>
         </is>
@@ -1595,51 +1608,51 @@
           <t>Jacket</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>2500</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>7272</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>1</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t xml:space="preserve">Sleevles + Hand Embroidery + Hand Painting </t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t xml:space="preserve">Off-White </t>
         </is>
@@ -1671,51 +1684,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Bamboo</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>3000</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>12121</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Long Shirt - Print + Medium Hand Embroidery</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Digital print + Hand Embroidery</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -1747,51 +1760,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Bamboo</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>3000</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>12121</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>1</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t xml:space="preserve">Long Shirt  Print + Upcycled Applique + Hand Embroidery </t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t xml:space="preserve">Black and White </t>
         </is>
@@ -1823,51 +1836,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Bamboo</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>1600</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>5995</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>1</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t xml:space="preserve">Flourscent Yellow </t>
         </is>
@@ -1899,46 +1912,46 @@
           <t>Jacket</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>10000</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>37373</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>1</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Sleevless + Upcycled + Half Embroidery</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t xml:space="preserve">Regular </t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -1970,41 +1983,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>300</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>4545</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>1</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t xml:space="preserve">Upcycled + Full Hand Embroidery  </t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2036,41 +2049,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>250</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>3535</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Upcycled + Medium Embroidery + Centre</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2102,41 +2115,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>250</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>3535</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>1</v>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2168,41 +2181,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>200</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>2002</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>1</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2234,41 +2247,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>150</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>1415</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>1</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2300,41 +2313,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>150</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>1112</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>Upcycled + Medium Embroidery  + Typography</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2366,41 +2379,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>100</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>888</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>1</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t xml:space="preserve">Upcycled + Print </t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Digital print + Hand Embroidery</t>
         </is>
@@ -2432,41 +2445,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>1000</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>4545</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>1</v>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>Hand Embroidery</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2498,41 +2511,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>200</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>1212</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>1</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>Hand Embroidery</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2564,41 +2577,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>1000</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>4545</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>Hand Embroidery</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand Embroidery </t>
         </is>
@@ -2630,41 +2643,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>70</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>555</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>1</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
@@ -2696,41 +2709,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>100</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>789</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
         <v>1</v>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
@@ -2762,41 +2775,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>70</v>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>555</v>
       </c>
-      <c r="J24" t="n">
+      <c r="K24" t="n">
         <v>1</v>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
@@ -2828,41 +2841,41 @@
           <t>Accessory</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Upcycled</t>
         </is>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>70</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>555</v>
       </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
         <v>1</v>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Hand Painting</t>
         </is>
@@ -2894,51 +2907,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>1200</v>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>2300</v>
       </c>
-      <c r="J26" t="n">
+      <c r="K26" t="n">
         <v>1</v>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="R26" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -2970,51 +2983,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>1200</v>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>2300</v>
       </c>
-      <c r="J27" t="n">
+      <c r="K27" t="n">
         <v>1</v>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="R27" t="inlineStr">
         <is>
           <t>Grey</t>
         </is>
@@ -3046,51 +3059,51 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>1200</v>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>2300</v>
       </c>
-      <c r="J28" t="n">
+      <c r="K28" t="n">
         <v>1</v>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="R28" t="inlineStr">
         <is>
           <t xml:space="preserve">Black and White </t>
         </is>
@@ -3122,46 +3135,46 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>1200</v>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>2300</v>
       </c>
-      <c r="J29" t="n">
+      <c r="K29" t="n">
         <v>1</v>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
@@ -3193,46 +3206,46 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>1200</v>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>2300</v>
       </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
         <v>1</v>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
@@ -3264,55 +3277,58 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Giza Cotton</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>1200</v>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>2300</v>
       </c>
-      <c r="J31" t="n">
+      <c r="K31" t="n">
         <v>1</v>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>Relaxed</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>Digital Print</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="M2:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active,Discontinued,Sold-out"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3325,7 +3341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3334,15 +3350,16 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3378,45 +3395,50 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>collection</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>geography</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>revenue</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>units_sold</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>discount_amount</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>returns_units</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>returns_value</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Product_name</t>
         </is>
@@ -3453,33 +3475,33 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>8000</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>4000</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Compliments</t>
         </is>
@@ -3516,33 +3538,33 @@
           <t>Shirt</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>10000</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>100</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>2</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Harm the harmonium</t>
         </is>
@@ -3579,18 +3601,18 @@
           <t>Handkerchief</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Black with face in the centre</t>
         </is>
@@ -3627,18 +3649,18 @@
           <t>Handkerchief</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -3661,7 +3683,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
+    </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Robust style_family lookup for letter-suffix SKUs; reshare workbook
- Dashboard: resolve REVENUE style_family via an INVENTORY sku->family lookup
  (not just stripping a numeric suffix), so SKUs ending in letters (e.g.
  HB1HE-HH) roll up to their family correctly; trim SKUs on both tabs.
- Reshared workbook from the studio's latest data: normalized SKU spacing,
  added size (Shirts=L, Accessories=Free Size, the two orders XS & L),
  added REVENUE.style_family via inventory lookup, fixed the 'MATERIALS '
  trailing-space tab name, refreshed How-to.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -18,7 +18,9 @@
     <sheet name="SKU_MATERIALS" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="ALERTS" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="TARGETS" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="How to" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Style-Family Naming" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Cust ID" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="How to" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,23 +44,14 @@
       <sz val="10"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="006B675E"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
       <sz val="11"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -68,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00161511"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFEDE6"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,19 +76,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -778,7 +762,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -798,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -835,27 +819,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>HB</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -867,124 +830,135 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:M32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Business Loomline — data guide</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>One record per row. Numbers plain (no ₹/commas). Dates as real dates. Use the dropdowns. Grey rows are examples — replace them.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>One record per row. Numbers plain. Dates as real dates. Use the dropdowns.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>THE KEY IDEA</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>KEY IDEA: sku = one physical piece (unique). style_family = the group (e.g. HB1HE). size is a piece attribute (each size = its own row + its own unit_cost).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>sku = one physical piece (unique, e.g. HB1HE-01).  style_family = the group (brand+collection+technique, e.g. HB1HE).</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>sku + style_family appear on INVENTORY, REVENUE and COSTS so everything links. size is on INVENTORY and REVENUE.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Size is a piece-level attribute: each size is its own INVENTORY row with its own unit_cost, so an L that costs more than an M is captured automatically.</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Both sku and style_family appear on INVENTORY, REVENUE and COSTS so everything links.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT: keep tab names EXACT (no trailing spaces) — MATERIALS, not 'MATERIALS '. Keep every sku spelling identical between INVENTORY and REVENUE.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TABS</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Still to fill: revenue amounts on the two blank handkerchief sales; the collection name (shows as '1'); sizes for the 2 jackets.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>INVENTORY — one row per finished piece; unique sku + style_family; size (XS…XXL/Free Size/Custom); unit_cost = make cost, unit_price = selling price.</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Jacket and accessory always stay separate — breakdowns use category, never merged by family.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>REVENUE — one row per sale; sku + style_family + size sold; revenue and units_sold.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>COSTS — one row per expense; cost_function; production spend gets a style_family so costs roll up per family.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>CHANNELS · CUSTOMERS · ALERTS · TARGETS — as before.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>MATERIALS — raw stock at a glance: status (In stock / Running low / Out of stock) + on_order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>SKU_MATERIALS (optional) — link a material to the pieces that use it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Jacket and accessory always stay separate — breakdowns use category/silhouette, never merged by family.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
         </is>
@@ -1205,7 +1179,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HB1PHE-01</t>
+          <t>HB1PHE-CP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1226,6 +1200,11 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1259,7 +1238,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Short Sleeve Shirt + Running Embroidery </t>
+          <t>Short Sleeve Shirt + Running Embroidery</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1281,7 +1260,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HB1HE-01</t>
+          <t>HB1HE-DY</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1302,6 +1281,11 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1335,7 +1319,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Long Sleeve Shirt  + Small Object Hand Embroidery  </t>
+          <t>Long Sleeve Shirt + Small Object Hand Embroidery</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1345,7 +1329,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1357,7 +1341,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HB1HE-02</t>
+          <t>HB1HE-PO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1380,6 +1364,11 @@
           <t>Shirt</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>#1</t>
@@ -1387,7 +1376,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed: Cotton + Linen </t>
+          <t>Mixed: Cotton + Linen</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -1411,7 +1400,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Short Sleeve + Long Crop Top + Medium Embroidery </t>
+          <t>Short Sleeve + Long Crop Top + Medium Embroidery</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1421,19 +1410,19 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t xml:space="preserve">White </t>
+          <t>White</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HB1HE-03</t>
+          <t>HB1HE-HH</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1454,6 +1443,11 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1497,19 +1491,19 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Off-White </t>
+          <t>Off-White</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HB1HE-04</t>
+          <t>HB1HE-SB</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1530,6 +1524,11 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1563,7 +1562,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Short Crop Shirt + Full Hand Embroidery  </t>
+          <t>Short Crop Shirt + Full Hand Embroidery</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1573,19 +1572,19 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t xml:space="preserve">White </t>
+          <t>White</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HBIHP-01</t>
+          <t>HBIHP-LB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1600,7 +1599,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lost Bubble - Hand Painting </t>
+          <t>Lost Bubble - Hand Painting</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1608,6 +1607,7 @@
           <t>Jacket</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>#1</t>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sleevles + Hand Embroidery + Hand Painting </t>
+          <t>Sleevles + Hand Embroidery + Hand Painting</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Off-White </t>
+          <t>Off-White</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HB1HE-05</t>
+          <t>HB1HE-CS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1682,6 +1682,11 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1737,7 +1742,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HB1HE-06</t>
+          <t>HB1HE-LM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1758,6 +1763,11 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1791,7 +1801,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Long Shirt  Print + Upcycled Applique + Hand Embroidery </t>
+          <t>Long Shirt Print + Upcycled Applique + Hand Embroidery</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1801,19 +1811,19 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black and White </t>
+          <t>Black and White</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HB1DP-01</t>
+          <t>HB1DP-PLY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1828,12 +1838,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unisex Plain </t>
+          <t xml:space="preserve">Unisex Plain - Flourescent Yellow </t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1867,7 +1882,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1882,14 +1897,14 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flourscent Yellow </t>
+          <t>Flourscent Yellow</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HB1JAHE-01</t>
+          <t>HB1JAHE-FF</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1912,6 +1927,7 @@
           <t>Jacket</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>#1</t>
@@ -1948,19 +1964,24 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regular </t>
+          <t>Regular</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Grey</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HB1UHE-01</t>
+          <t>HB1UHE-H1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1981,6 +2002,11 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2014,19 +2040,24 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upcycled + Full Hand Embroidery  </t>
+          <t>Upcycled + Full Hand Embroidery</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Black and White</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HB1UHE-02</t>
+          <t>HB1UHE-H2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2047,6 +2078,11 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2085,14 +2121,19 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>White</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HB1UHE-03</t>
+          <t>HB1UHE-H3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2113,6 +2154,11 @@
       <c r="E14" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2146,19 +2192,24 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
+          <t>Upcycled + Medium Embroidery + Boder</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>White</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HB1UHE-04</t>
+          <t>HB1UHE-H4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2179,6 +2230,11 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2212,19 +2268,24 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
+          <t>Upcycled + Medium Embroidery + Boder</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Yellow</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HB1UP-01</t>
+          <t>HB1UP-H5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2245,6 +2306,11 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2278,19 +2344,24 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upcycled + Medium Embroidery + Boder </t>
+          <t>Upcycled + Medium Embroidery + Boder</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Black and White</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HB1UP-02</t>
+          <t>HB1UP-H6</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2311,6 +2382,11 @@
       <c r="E17" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2344,19 +2420,24 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Upcycled + Medium Embroidery  + Typography</t>
+          <t>Upcycled + Medium Embroidery + Typography</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Black</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HB1UHE-05</t>
+          <t>HB1UHE-H7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2377,6 +2458,11 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2410,7 +2496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upcycled + Print </t>
+          <t>Upcycled + Print</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -2422,7 +2508,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HB1UHE-06</t>
+          <t>HB1UHE-PS1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2443,6 +2529,11 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2481,14 +2572,14 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HB1UHE-07</t>
+          <t>HB1UHE-PS2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2509,6 +2600,11 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2547,14 +2643,14 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HB1UHE-08</t>
+          <t>HB1UHE-PS3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2575,6 +2671,11 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2613,14 +2714,14 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand Embroidery </t>
+          <t>Hand Embroidery</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HB1UHP-01</t>
+          <t>HB1UHP-BD1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2641,6 +2742,11 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2686,7 +2792,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HB1UHP-02</t>
+          <t>HB1UHP-BD2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2707,6 +2813,11 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2752,7 +2863,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HB1UHP-03</t>
+          <t>HB1UHP-BD3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2773,6 +2884,11 @@
       <c r="E24" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2818,7 +2934,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HB1UHP-04</t>
+          <t>HB1UHP-BD4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2839,6 +2955,11 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2884,7 +3005,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PS1DP-01</t>
+          <t>PS1DP-REF</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2905,6 +3026,11 @@
       <c r="E26" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2938,7 +3064,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2960,7 +3086,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PS1DP-02</t>
+          <t>PS1DP-GYF</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2981,6 +3107,11 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3014,7 +3145,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3036,7 +3167,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PS1DP-03</t>
+          <t>PS1DP-BWP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3057,6 +3188,11 @@
       <c r="E28" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3090,7 +3226,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3105,14 +3241,14 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black and White </t>
+          <t>Black and White</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PS1DP-04</t>
+          <t>PS1DP-LCC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3133,6 +3269,11 @@
       <c r="E29" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3166,7 +3307,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3183,7 +3324,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PS1DP-05</t>
+          <t>PS1DP-BLM</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3204,6 +3345,11 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3237,7 +3383,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3254,7 +3400,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PS1DP-06</t>
+          <t>PS1DP-TPS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3275,6 +3421,11 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3308,7 +3459,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Half Sleeve + Digital Print One Colour </t>
+          <t>Half Sleeve + Digital Print One Colour</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3324,11 +3475,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
+    </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active,Discontinued,Sold-out"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3341,7 +3492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3457,14 +3608,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>HB1PHE-CP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>HB1PHE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HB1PHE</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Retail</t>
@@ -3473,6 +3624,11 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>XS</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -3498,8 +3654,10 @@
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="n">
-        <v>1</v>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>HB002</t>
+        </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -3520,14 +3678,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>HB1HE-HH</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>HB1HE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>HB1HE</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Retail</t>
@@ -3536,6 +3694,11 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Shirt</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -3561,8 +3724,10 @@
       <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" t="n">
-        <v>2</v>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>HB001</t>
+        </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -3583,14 +3748,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>HB1UHE-H7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>HB1UHE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>HB1UHE</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Retail</t>
@@ -3599,6 +3764,11 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Handkerchief</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3631,14 +3801,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>HB1UHE-H7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>HB1UHE</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>HB1UHE</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Retail</t>
@@ -3647,6 +3817,11 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Handkerchief</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Free Size</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -3663,22 +3838,6 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>TBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="D6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Integrate product name </t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Integrate unit price</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3936,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3822,7 +3981,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>06/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3867,7 +4026,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3912,7 +4071,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>08/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3957,7 +4116,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>09/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4002,7 +4161,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4047,7 +4206,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4092,7 +4251,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4137,7 +4296,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4182,7 +4341,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4227,7 +4386,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>15/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4267,7 +4426,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>16/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4317,7 +4476,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>17/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4367,7 +4526,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18/01/2026</t>
+          <t>04/01/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4412,7 +4571,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>19/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4457,7 +4616,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>20/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4492,7 +4651,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4527,7 +4686,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>22/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4562,7 +4721,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>23/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4597,7 +4756,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>24/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4632,7 +4791,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4667,7 +4826,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>26/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4702,7 +4861,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>27/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4737,7 +4896,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>28/01/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4772,7 +4931,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4809,7 +4968,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>30/01/2026</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4854,7 +5013,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>31/01/2026</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5205,296 +5364,244 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Bamboo fabric</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Fabric</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>metre</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>In stock</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Fabriclore</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Linen (Jaipur)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Fabric</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>metre</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Out of stock</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>05/08/2026</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Bapu Bazar</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>for longline shirts</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Black thread</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Thread</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>spool</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>In stock</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>White thread</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Thread</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>spool</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Running low</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Fabric paint — red</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Paint</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>jar</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Running low</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Jaipur</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Wooden buttons</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Button</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>piece</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>In stock</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Delhi</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Poly mailers</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Packaging</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>piece</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Running low</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>shipping</t>
         </is>
@@ -5563,75 +5670,74 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>HB1HE-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Bamboo fabric</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>1.5</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>metre</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>shirt body</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>HB1HE-01</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Black thread</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" t="n">
         <v>0.2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>spool</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>embroidery</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>HB1UHP-01</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Wooden buttons</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>piece</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final workbook: add REVENUE.unit_cost + Sample status/stage for made-to-order
Adds the made-to-order + sample-cost columns/options to the studio workbook:
- REVENUE.unit_cost (per-order make-cost, for true custom-order margin)
- INVENTORY.status dropdown gains Sample / Made to order
- COSTS.cost_stage dropdown gains Sample (samples logged as R&D cost)
- How-to explains samples-as-cost and per-order unit_cost.
Dashboard wiring to consume these follows once the data is in.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,10 @@
     </font>
     <font>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -76,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -85,6 +89,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -893,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -909,7 +916,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>One record per row. Numbers plain. Dates as real dates. Use the dropdowns.</t>
+          <t>One record per row. Numbers plain. Dates as real dates. Use the dropdowns. Keep tab names EXACT (no trailing spaces).</t>
         </is>
       </c>
     </row>
@@ -919,46 +926,53 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>KEY IDEA: sku = one physical piece (unique). style_family = the group (e.g. HB1HE). size is a piece attribute (each size = its own row + its own unit_cost).</t>
+          <t>KEYS: sku = one physical piece (unique). style_family = the group (e.g. HB1HE). size = piece attribute (each size = own row + own cost).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>sku + style_family appear on INVENTORY, REVENUE and COSTS so everything links. size is on INVENTORY and REVENUE.</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MADE-TO-ORDER &amp; SAMPLES</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>IMPORTANT: keep tab names EXACT (no trailing spaces) — MATERIALS, not 'MATERIALS '. Keep every sku spelling identical between INVENTORY and REVENUE.</t>
+          <t>Samples are a real COST: log the sample's make-cost in COSTS with cost_stage = Sample (shows in R&amp;D). In INVENTORY mark the showcase piece status = Sample.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Custom orders: each REVENUE row gets size + unit_cost = what THAT order cost to make (size drives cost). Margin per order = revenue − unit_cost.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Still to fill: revenue amounts on the two blank handkerchief sales; the collection name (shows as '1'); sizes for the 2 jackets.</t>
+          <t>So: sample = expensed cost; order = revenue minus its own make-cost. No double counting.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Jacket and accessory always stay separate — breakdowns use category, never merged by family.</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Still to fill: revenue amounts on the two blank handkerchief sales; a real collection name (shows as '1'); jacket sizes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
         </is>
@@ -3479,7 +3493,7 @@
       <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Active,Discontinued,Sold-out"</formula1>
+      <formula1>"Active,Sample,Made to order,Discontinued,Sold-out"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3492,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3505,12 +3519,13 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3566,30 +3581,35 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>unit_cost</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>units_sold</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>discount_amount</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>returns_units</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>returns_value</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Product_name</t>
         </is>
@@ -3642,24 +3662,24 @@
       <c r="J2" t="n">
         <v>8000</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>4000</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>HB002</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Compliments</t>
         </is>
@@ -3712,24 +3732,24 @@
       <c r="J3" t="n">
         <v>10000</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>1</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>100</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>HB001</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Harm the harmonium</t>
         </is>
@@ -3779,10 +3799,10 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>1</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Black with face in the centre</t>
         </is>
@@ -3832,10 +3852,10 @@
           <t>Mumbai</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>1</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
@@ -5051,9 +5071,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Product,Marketing &amp; brand,Overheads"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Experiment,Sample,Final production,—"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Automate MATERIALS + SKU_MATERIALS (auto-deduct, rate, cost, family)
Formula-driven workbook so the sheet maintains itself:
- MATERIALS: rate = total_cost/qty_bought; quantity_on_hand = qty_bought −
  SUMIF(usage); status auto (In stock/Running low/Out).
- SKU_MATERIALS usage log: pick sku + material from dropdowns → style_family,
  unit, rate and cost (qty×rate) auto-fill; logging a use auto-deducts from
  MATERIALS on-hand and captures R&D vs Production per row.
- Dropdowns: sku (from INVENTORY), material (from MATERIALS), use_type.
- Formulas pre-filled down 80 rows with blank-guards; auto columns tinted.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6VD4ZFysqCKpWchDyCKBD
</commit_message>
<xml_diff>
--- a/docs/Business Loomline — updated.xlsx
+++ b/docs/Business Loomline — updated.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,11 @@
     <font>
       <b val="1"/>
       <color rgb="00F3F2ED"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B675E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -55,7 +60,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +70,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00161511"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEDE6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,18 +95,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -903,78 +920,82 @@
   <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="118" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Business Loomline — data guide</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Business Loomline — data guide + automation</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>One record per row. Numbers plain. Dates as real dates. Use the dropdowns. Keep tab names EXACT (no trailing spaces).</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Blue-tinted columns are AUTOMATIC (formulas) — don't type in them. Fill the rest; use the dropdowns.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
+      <c r="A3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>KEYS: sku = one physical piece (unique). style_family = the group (e.g. HB1HE). size = piece attribute (each size = own row + own cost).</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>MATERIALS — buy once, it tracks the rest</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Type: material, category, unit, qty_bought, total_cost, reorder_level. Auto: rate (cost/qty), quantity_on_hand (bought − used), status.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>MADE-TO-ORDER &amp; SAMPLES</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SKU_MATERIALS — log each fabric use, it does the maths</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Samples are a real COST: log the sample's make-cost in COSTS with cost_stage = Sample (shows in R&amp;D). In INVENTORY mark the showcase piece status = Sample.</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Type: date, sku (dropdown), material (dropdown), use_type (R&amp;D/Production), qty_used. Auto: style_family, unit, rate, cost.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Custom orders: each REVENUE row gets size + unit_cost = what THAT order cost to make (size drives cost). Margin per order = revenue − unit_cost.</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Logging a use auto-deducts from MATERIALS.quantity_on_hand; R&amp;D vs Production is captured per row.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>So: sample = expensed cost; order = revenue minus its own make-cost. No double counting.</t>
-        </is>
-      </c>
+      <c r="A9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Money rule: the fabric PURCHASE is the expense — log it once in COSTS. MATERIALS/SKU_MATERIALS track metres + per-piece cost (reference), not a second expense.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Still to fill: revenue amounts on the two blank handkerchief sales; a real collection name (shows as '1'); jacket sizes.</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Keep tab names EXACT and sku spelling identical across tabs so dropdowns/lookups work.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Full model &amp; formulas: docs/business-math-data-model.md</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Full model: docs/business-math-data-model.md</t>
         </is>
       </c>
     </row>
@@ -3489,10 +3510,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active,Sample,Made to order,Discontinued,Sold-out"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3863,10 +3884,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"XS,S,M,L,XL,XXL,Free Size,Custom"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5072,13 +5093,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HB1DP,HB1HE,HB1JAHE,HB1PHE,HB1UHE,HB1UHP,HB1UP,HBIHP,PS1DP"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Product,Marketing &amp; brand,Overheads"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Experiment,Sample,Final production,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5322,19 +5343,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5355,76 +5379,112 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>qty_bought</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>total_cost</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>quantity_on_hand</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>reorder_level</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>on_order</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>expected_date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>supplier</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bamboo fabric</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bamboo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Fabric</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>metre</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>In stock</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="D2" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>8100</v>
+      </c>
+      <c r="F2" s="3">
+        <f>IF($D2&gt;0,$E2/$D2,"")</f>
+        <v/>
+      </c>
+      <c r="G2" s="3">
+        <f>IF($D2="","",$D2-SUMIF(SKU_MATERIALS!$D:$D,$A2,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="3">
+        <f>IF($G2="","",IF($G2&lt;=0,"Out of stock",IF(AND($H2&lt;&gt;"",$G2&lt;=$H2),"Running low","In stock")))</f>
+        <v/>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Fabriclore</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>example — 15 m bought</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Linen (Jaipur)</t>
+          <t>100% Linen</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5437,214 +5497,1253 @@
           <t>metre</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Out of stock</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>08/05/2026</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Bapu Bazar</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>for longline shirts</t>
-        </is>
+      <c r="F3" s="3">
+        <f>IF($D3&gt;0,$E3/$D3,"")</f>
+        <v/>
+      </c>
+      <c r="G3" s="3">
+        <f>IF($D3="","",$D3-SUMIF(SKU_MATERIALS!$D:$D,$A3,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" s="3">
+        <f>IF($G3="","",IF($G3&lt;=0,"Out of stock",IF(AND($H3&lt;&gt;"",$G3&lt;=$H3),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Black thread</t>
+          <t>Mixed: Cotton + Linen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thread</t>
+          <t>Fabric</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>spool</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>In stock</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
+          <t>metre</t>
+        </is>
+      </c>
+      <c r="F4" s="3">
+        <f>IF($D4&gt;0,$E4/$D4,"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="3">
+        <f>IF($D4="","",$D4-SUMIF(SKU_MATERIALS!$D:$D,$A4,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="3">
+        <f>IF($G4="","",IF($G4&lt;=0,"Out of stock",IF(AND($H4&lt;&gt;"",$G4&lt;=$H4),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>White thread</t>
+          <t>Upcycled</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Thread</t>
+          <t>Fabric</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>spool</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Running low</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
+          <t>metre</t>
+        </is>
+      </c>
+      <c r="F5" s="3">
+        <f>IF($D5&gt;0,$E5/$D5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="3">
+        <f>IF($D5="","",$D5-SUMIF(SKU_MATERIALS!$D:$D,$A5,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="3">
+        <f>IF($G5="","",IF($G5&lt;=0,"Out of stock",IF(AND($H5&lt;&gt;"",$G5&lt;=$H5),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fabric paint — red</t>
+          <t>Giza Cotton</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paint</t>
+          <t>Fabric</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>jar</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Running low</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Jaipur</t>
-        </is>
+          <t>metre</t>
+        </is>
+      </c>
+      <c r="F6" s="3">
+        <f>IF($D6&gt;0,$E6/$D6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="3">
+        <f>IF($D6="","",$D6-SUMIF(SKU_MATERIALS!$D:$D,$A6,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" s="3">
+        <f>IF($G6="","",IF($G6&lt;=0,"Out of stock",IF(AND($H6&lt;&gt;"",$G6&lt;=$H6),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wooden buttons</t>
+          <t>Black thread</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>Thread</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>piece</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>In stock</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
+          <t>spool</t>
+        </is>
+      </c>
+      <c r="F7" s="3">
+        <f>IF($D7&gt;0,$E7/$D7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="3">
+        <f>IF($D7="","",$D7-SUMIF(SKU_MATERIALS!$D:$D,$A7,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="3">
+        <f>IF($G7="","",IF($G7&lt;=0,"Out of stock",IF(AND($H7&lt;&gt;"",$G7&lt;=$H7),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>White thread</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Thread</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>spool</t>
+        </is>
+      </c>
+      <c r="F8" s="3">
+        <f>IF($D8&gt;0,$E8/$D8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="3">
+        <f>IF($D8="","",$D8-SUMIF(SKU_MATERIALS!$D:$D,$A8,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="3">
+        <f>IF($G8="","",IF($G8&lt;=0,"Out of stock",IF(AND($H8&lt;&gt;"",$G8&lt;=$H8),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Wooden buttons</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="F9" s="3">
+        <f>IF($D9&gt;0,$E9/$D9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>IF($D9="","",$D9-SUMIF(SKU_MATERIALS!$D:$D,$A9,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" s="3">
+        <f>IF($G9="","",IF($G9&lt;=0,"Out of stock",IF(AND($H9&lt;&gt;"",$G9&lt;=$H9),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fabric paint — red</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paint</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>jar</t>
+        </is>
+      </c>
+      <c r="F10" s="3">
+        <f>IF($D10&gt;0,$E10/$D10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="3">
+        <f>IF($D10="","",$D10-SUMIF(SKU_MATERIALS!$D:$D,$A10,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="3">
+        <f>IF($G10="","",IF($G10&lt;=0,"Out of stock",IF(AND($H10&lt;&gt;"",$G10&lt;=$H10),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Poly mailers</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Packaging</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>piece</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Running low</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
+      <c r="F11" s="3">
+        <f>IF($D11&gt;0,$E11/$D11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>IF($D11="","",$D11-SUMIF(SKU_MATERIALS!$D:$D,$A11,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" s="3">
+        <f>IF($G11="","",IF($G11&lt;=0,"Out of stock",IF(AND($H11&lt;&gt;"",$G11&lt;=$H11),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="F12" s="3">
+        <f>IF($D12&gt;0,$E12/$D12,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="3">
+        <f>IF($D12="","",$D12-SUMIF(SKU_MATERIALS!$D:$D,$A12,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I12" s="3">
+        <f>IF($G12="","",IF($G12&lt;=0,"Out of stock",IF(AND($H12&lt;&gt;"",$G12&lt;=$H12),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="F13" s="3">
+        <f>IF($D13&gt;0,$E13/$D13,"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="3">
+        <f>IF($D13="","",$D13-SUMIF(SKU_MATERIALS!$D:$D,$A13,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I13" s="3">
+        <f>IF($G13="","",IF($G13&lt;=0,"Out of stock",IF(AND($H13&lt;&gt;"",$G13&lt;=$H13),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" s="3">
+        <f>IF($D14&gt;0,$E14/$D14,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="3">
+        <f>IF($D14="","",$D14-SUMIF(SKU_MATERIALS!$D:$D,$A14,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I14" s="3">
+        <f>IF($G14="","",IF($G14&lt;=0,"Out of stock",IF(AND($H14&lt;&gt;"",$G14&lt;=$H14),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="F15" s="3">
+        <f>IF($D15&gt;0,$E15/$D15,"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="3">
+        <f>IF($D15="","",$D15-SUMIF(SKU_MATERIALS!$D:$D,$A15,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I15" s="3">
+        <f>IF($G15="","",IF($G15&lt;=0,"Out of stock",IF(AND($H15&lt;&gt;"",$G15&lt;=$H15),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="F16" s="3">
+        <f>IF($D16&gt;0,$E16/$D16,"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="3">
+        <f>IF($D16="","",$D16-SUMIF(SKU_MATERIALS!$D:$D,$A16,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I16" s="3">
+        <f>IF($G16="","",IF($G16&lt;=0,"Out of stock",IF(AND($H16&lt;&gt;"",$G16&lt;=$H16),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="F17" s="3">
+        <f>IF($D17&gt;0,$E17/$D17,"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="3">
+        <f>IF($D17="","",$D17-SUMIF(SKU_MATERIALS!$D:$D,$A17,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I17" s="3">
+        <f>IF($G17="","",IF($G17&lt;=0,"Out of stock",IF(AND($H17&lt;&gt;"",$G17&lt;=$H17),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="F18" s="3">
+        <f>IF($D18&gt;0,$E18/$D18,"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="3">
+        <f>IF($D18="","",$D18-SUMIF(SKU_MATERIALS!$D:$D,$A18,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I18" s="3">
+        <f>IF($G18="","",IF($G18&lt;=0,"Out of stock",IF(AND($H18&lt;&gt;"",$G18&lt;=$H18),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="F19" s="3">
+        <f>IF($D19&gt;0,$E19/$D19,"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="3">
+        <f>IF($D19="","",$D19-SUMIF(SKU_MATERIALS!$D:$D,$A19,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I19" s="3">
+        <f>IF($G19="","",IF($G19&lt;=0,"Out of stock",IF(AND($H19&lt;&gt;"",$G19&lt;=$H19),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="F20" s="3">
+        <f>IF($D20&gt;0,$E20/$D20,"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="3">
+        <f>IF($D20="","",$D20-SUMIF(SKU_MATERIALS!$D:$D,$A20,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I20" s="3">
+        <f>IF($G20="","",IF($G20&lt;=0,"Out of stock",IF(AND($H20&lt;&gt;"",$G20&lt;=$H20),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="F21" s="3">
+        <f>IF($D21&gt;0,$E21/$D21,"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="3">
+        <f>IF($D21="","",$D21-SUMIF(SKU_MATERIALS!$D:$D,$A21,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I21" s="3">
+        <f>IF($G21="","",IF($G21&lt;=0,"Out of stock",IF(AND($H21&lt;&gt;"",$G21&lt;=$H21),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="F22" s="3">
+        <f>IF($D22&gt;0,$E22/$D22,"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="3">
+        <f>IF($D22="","",$D22-SUMIF(SKU_MATERIALS!$D:$D,$A22,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I22" s="3">
+        <f>IF($G22="","",IF($G22&lt;=0,"Out of stock",IF(AND($H22&lt;&gt;"",$G22&lt;=$H22),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="F23" s="3">
+        <f>IF($D23&gt;0,$E23/$D23,"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="3">
+        <f>IF($D23="","",$D23-SUMIF(SKU_MATERIALS!$D:$D,$A23,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I23" s="3">
+        <f>IF($G23="","",IF($G23&lt;=0,"Out of stock",IF(AND($H23&lt;&gt;"",$G23&lt;=$H23),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="F24" s="3">
+        <f>IF($D24&gt;0,$E24/$D24,"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="3">
+        <f>IF($D24="","",$D24-SUMIF(SKU_MATERIALS!$D:$D,$A24,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I24" s="3">
+        <f>IF($G24="","",IF($G24&lt;=0,"Out of stock",IF(AND($H24&lt;&gt;"",$G24&lt;=$H24),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="3">
+        <f>IF($D25&gt;0,$E25/$D25,"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="3">
+        <f>IF($D25="","",$D25-SUMIF(SKU_MATERIALS!$D:$D,$A25,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I25" s="3">
+        <f>IF($G25="","",IF($G25&lt;=0,"Out of stock",IF(AND($H25&lt;&gt;"",$G25&lt;=$H25),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="F26" s="3">
+        <f>IF($D26&gt;0,$E26/$D26,"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="3">
+        <f>IF($D26="","",$D26-SUMIF(SKU_MATERIALS!$D:$D,$A26,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I26" s="3">
+        <f>IF($G26="","",IF($G26&lt;=0,"Out of stock",IF(AND($H26&lt;&gt;"",$G26&lt;=$H26),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="3">
+        <f>IF($D27&gt;0,$E27/$D27,"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="3">
+        <f>IF($D27="","",$D27-SUMIF(SKU_MATERIALS!$D:$D,$A27,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I27" s="3">
+        <f>IF($G27="","",IF($G27&lt;=0,"Out of stock",IF(AND($H27&lt;&gt;"",$G27&lt;=$H27),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="F28" s="3">
+        <f>IF($D28&gt;0,$E28/$D28,"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="3">
+        <f>IF($D28="","",$D28-SUMIF(SKU_MATERIALS!$D:$D,$A28,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I28" s="3">
+        <f>IF($G28="","",IF($G28&lt;=0,"Out of stock",IF(AND($H28&lt;&gt;"",$G28&lt;=$H28),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="F29" s="3">
+        <f>IF($D29&gt;0,$E29/$D29,"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="3">
+        <f>IF($D29="","",$D29-SUMIF(SKU_MATERIALS!$D:$D,$A29,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I29" s="3">
+        <f>IF($G29="","",IF($G29&lt;=0,"Out of stock",IF(AND($H29&lt;&gt;"",$G29&lt;=$H29),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="F30" s="3">
+        <f>IF($D30&gt;0,$E30/$D30,"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="3">
+        <f>IF($D30="","",$D30-SUMIF(SKU_MATERIALS!$D:$D,$A30,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I30" s="3">
+        <f>IF($G30="","",IF($G30&lt;=0,"Out of stock",IF(AND($H30&lt;&gt;"",$G30&lt;=$H30),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="F31" s="3">
+        <f>IF($D31&gt;0,$E31/$D31,"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="3">
+        <f>IF($D31="","",$D31-SUMIF(SKU_MATERIALS!$D:$D,$A31,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I31" s="3">
+        <f>IF($G31="","",IF($G31&lt;=0,"Out of stock",IF(AND($H31&lt;&gt;"",$G31&lt;=$H31),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="F32" s="3">
+        <f>IF($D32&gt;0,$E32/$D32,"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="3">
+        <f>IF($D32="","",$D32-SUMIF(SKU_MATERIALS!$D:$D,$A32,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I32" s="3">
+        <f>IF($G32="","",IF($G32&lt;=0,"Out of stock",IF(AND($H32&lt;&gt;"",$G32&lt;=$H32),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="F33" s="3">
+        <f>IF($D33&gt;0,$E33/$D33,"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="3">
+        <f>IF($D33="","",$D33-SUMIF(SKU_MATERIALS!$D:$D,$A33,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I33" s="3">
+        <f>IF($G33="","",IF($G33&lt;=0,"Out of stock",IF(AND($H33&lt;&gt;"",$G33&lt;=$H33),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="F34" s="3">
+        <f>IF($D34&gt;0,$E34/$D34,"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="3">
+        <f>IF($D34="","",$D34-SUMIF(SKU_MATERIALS!$D:$D,$A34,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I34" s="3">
+        <f>IF($G34="","",IF($G34&lt;=0,"Out of stock",IF(AND($H34&lt;&gt;"",$G34&lt;=$H34),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="F35" s="3">
+        <f>IF($D35&gt;0,$E35/$D35,"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="3">
+        <f>IF($D35="","",$D35-SUMIF(SKU_MATERIALS!$D:$D,$A35,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I35" s="3">
+        <f>IF($G35="","",IF($G35&lt;=0,"Out of stock",IF(AND($H35&lt;&gt;"",$G35&lt;=$H35),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="F36" s="3">
+        <f>IF($D36&gt;0,$E36/$D36,"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="3">
+        <f>IF($D36="","",$D36-SUMIF(SKU_MATERIALS!$D:$D,$A36,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I36" s="3">
+        <f>IF($G36="","",IF($G36&lt;=0,"Out of stock",IF(AND($H36&lt;&gt;"",$G36&lt;=$H36),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="F37" s="3">
+        <f>IF($D37&gt;0,$E37/$D37,"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="3">
+        <f>IF($D37="","",$D37-SUMIF(SKU_MATERIALS!$D:$D,$A37,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I37" s="3">
+        <f>IF($G37="","",IF($G37&lt;=0,"Out of stock",IF(AND($H37&lt;&gt;"",$G37&lt;=$H37),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="3">
+        <f>IF($D38&gt;0,$E38/$D38,"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="3">
+        <f>IF($D38="","",$D38-SUMIF(SKU_MATERIALS!$D:$D,$A38,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I38" s="3">
+        <f>IF($G38="","",IF($G38&lt;=0,"Out of stock",IF(AND($H38&lt;&gt;"",$G38&lt;=$H38),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="F39" s="3">
+        <f>IF($D39&gt;0,$E39/$D39,"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="3">
+        <f>IF($D39="","",$D39-SUMIF(SKU_MATERIALS!$D:$D,$A39,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I39" s="3">
+        <f>IF($G39="","",IF($G39&lt;=0,"Out of stock",IF(AND($H39&lt;&gt;"",$G39&lt;=$H39),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="F40" s="3">
+        <f>IF($D40&gt;0,$E40/$D40,"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="3">
+        <f>IF($D40="","",$D40-SUMIF(SKU_MATERIALS!$D:$D,$A40,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I40" s="3">
+        <f>IF($G40="","",IF($G40&lt;=0,"Out of stock",IF(AND($H40&lt;&gt;"",$G40&lt;=$H40),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="F41" s="3">
+        <f>IF($D41&gt;0,$E41/$D41,"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="3">
+        <f>IF($D41="","",$D41-SUMIF(SKU_MATERIALS!$D:$D,$A41,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I41" s="3">
+        <f>IF($G41="","",IF($G41&lt;=0,"Out of stock",IF(AND($H41&lt;&gt;"",$G41&lt;=$H41),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="F42" s="3">
+        <f>IF($D42&gt;0,$E42/$D42,"")</f>
+        <v/>
+      </c>
+      <c r="G42" s="3">
+        <f>IF($D42="","",$D42-SUMIF(SKU_MATERIALS!$D:$D,$A42,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I42" s="3">
+        <f>IF($G42="","",IF($G42&lt;=0,"Out of stock",IF(AND($H42&lt;&gt;"",$G42&lt;=$H42),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="F43" s="3">
+        <f>IF($D43&gt;0,$E43/$D43,"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="3">
+        <f>IF($D43="","",$D43-SUMIF(SKU_MATERIALS!$D:$D,$A43,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I43" s="3">
+        <f>IF($G43="","",IF($G43&lt;=0,"Out of stock",IF(AND($H43&lt;&gt;"",$G43&lt;=$H43),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="F44" s="3">
+        <f>IF($D44&gt;0,$E44/$D44,"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="3">
+        <f>IF($D44="","",$D44-SUMIF(SKU_MATERIALS!$D:$D,$A44,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I44" s="3">
+        <f>IF($G44="","",IF($G44&lt;=0,"Out of stock",IF(AND($H44&lt;&gt;"",$G44&lt;=$H44),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="F45" s="3">
+        <f>IF($D45&gt;0,$E45/$D45,"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="3">
+        <f>IF($D45="","",$D45-SUMIF(SKU_MATERIALS!$D:$D,$A45,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I45" s="3">
+        <f>IF($G45="","",IF($G45&lt;=0,"Out of stock",IF(AND($H45&lt;&gt;"",$G45&lt;=$H45),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="F46" s="3">
+        <f>IF($D46&gt;0,$E46/$D46,"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="3">
+        <f>IF($D46="","",$D46-SUMIF(SKU_MATERIALS!$D:$D,$A46,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I46" s="3">
+        <f>IF($G46="","",IF($G46&lt;=0,"Out of stock",IF(AND($H46&lt;&gt;"",$G46&lt;=$H46),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="F47" s="3">
+        <f>IF($D47&gt;0,$E47/$D47,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="3">
+        <f>IF($D47="","",$D47-SUMIF(SKU_MATERIALS!$D:$D,$A47,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I47" s="3">
+        <f>IF($G47="","",IF($G47&lt;=0,"Out of stock",IF(AND($H47&lt;&gt;"",$G47&lt;=$H47),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="F48" s="3">
+        <f>IF($D48&gt;0,$E48/$D48,"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="3">
+        <f>IF($D48="","",$D48-SUMIF(SKU_MATERIALS!$D:$D,$A48,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I48" s="3">
+        <f>IF($G48="","",IF($G48&lt;=0,"Out of stock",IF(AND($H48&lt;&gt;"",$G48&lt;=$H48),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="F49" s="3">
+        <f>IF($D49&gt;0,$E49/$D49,"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="3">
+        <f>IF($D49="","",$D49-SUMIF(SKU_MATERIALS!$D:$D,$A49,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I49" s="3">
+        <f>IF($G49="","",IF($G49&lt;=0,"Out of stock",IF(AND($H49&lt;&gt;"",$G49&lt;=$H49),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="F50" s="3">
+        <f>IF($D50&gt;0,$E50/$D50,"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="3">
+        <f>IF($D50="","",$D50-SUMIF(SKU_MATERIALS!$D:$D,$A50,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I50" s="3">
+        <f>IF($G50="","",IF($G50&lt;=0,"Out of stock",IF(AND($H50&lt;&gt;"",$G50&lt;=$H50),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="F51" s="3">
+        <f>IF($D51&gt;0,$E51/$D51,"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="3">
+        <f>IF($D51="","",$D51-SUMIF(SKU_MATERIALS!$D:$D,$A51,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I51" s="3">
+        <f>IF($G51="","",IF($G51&lt;=0,"Out of stock",IF(AND($H51&lt;&gt;"",$G51&lt;=$H51),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="F52" s="3">
+        <f>IF($D52&gt;0,$E52/$D52,"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="3">
+        <f>IF($D52="","",$D52-SUMIF(SKU_MATERIALS!$D:$D,$A52,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I52" s="3">
+        <f>IF($G52="","",IF($G52&lt;=0,"Out of stock",IF(AND($H52&lt;&gt;"",$G52&lt;=$H52),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="F53" s="3">
+        <f>IF($D53&gt;0,$E53/$D53,"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="3">
+        <f>IF($D53="","",$D53-SUMIF(SKU_MATERIALS!$D:$D,$A53,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I53" s="3">
+        <f>IF($G53="","",IF($G53&lt;=0,"Out of stock",IF(AND($H53&lt;&gt;"",$G53&lt;=$H53),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="F54" s="3">
+        <f>IF($D54&gt;0,$E54/$D54,"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="3">
+        <f>IF($D54="","",$D54-SUMIF(SKU_MATERIALS!$D:$D,$A54,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I54" s="3">
+        <f>IF($G54="","",IF($G54&lt;=0,"Out of stock",IF(AND($H54&lt;&gt;"",$G54&lt;=$H54),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="F55" s="3">
+        <f>IF($D55&gt;0,$E55/$D55,"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="3">
+        <f>IF($D55="","",$D55-SUMIF(SKU_MATERIALS!$D:$D,$A55,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I55" s="3">
+        <f>IF($G55="","",IF($G55&lt;=0,"Out of stock",IF(AND($H55&lt;&gt;"",$G55&lt;=$H55),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="F56" s="3">
+        <f>IF($D56&gt;0,$E56/$D56,"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="3">
+        <f>IF($D56="","",$D56-SUMIF(SKU_MATERIALS!$D:$D,$A56,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I56" s="3">
+        <f>IF($G56="","",IF($G56&lt;=0,"Out of stock",IF(AND($H56&lt;&gt;"",$G56&lt;=$H56),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="F57" s="3">
+        <f>IF($D57&gt;0,$E57/$D57,"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="3">
+        <f>IF($D57="","",$D57-SUMIF(SKU_MATERIALS!$D:$D,$A57,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I57" s="3">
+        <f>IF($G57="","",IF($G57&lt;=0,"Out of stock",IF(AND($H57&lt;&gt;"",$G57&lt;=$H57),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="F58" s="3">
+        <f>IF($D58&gt;0,$E58/$D58,"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="3">
+        <f>IF($D58="","",$D58-SUMIF(SKU_MATERIALS!$D:$D,$A58,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I58" s="3">
+        <f>IF($G58="","",IF($G58&lt;=0,"Out of stock",IF(AND($H58&lt;&gt;"",$G58&lt;=$H58),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="F59" s="3">
+        <f>IF($D59&gt;0,$E59/$D59,"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="3">
+        <f>IF($D59="","",$D59-SUMIF(SKU_MATERIALS!$D:$D,$A59,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I59" s="3">
+        <f>IF($G59="","",IF($G59&lt;=0,"Out of stock",IF(AND($H59&lt;&gt;"",$G59&lt;=$H59),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="F60" s="3">
+        <f>IF($D60&gt;0,$E60/$D60,"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="3">
+        <f>IF($D60="","",$D60-SUMIF(SKU_MATERIALS!$D:$D,$A60,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I60" s="3">
+        <f>IF($G60="","",IF($G60&lt;=0,"Out of stock",IF(AND($H60&lt;&gt;"",$G60&lt;=$H60),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="F61" s="3">
+        <f>IF($D61&gt;0,$E61/$D61,"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="3">
+        <f>IF($D61="","",$D61-SUMIF(SKU_MATERIALS!$D:$D,$A61,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I61" s="3">
+        <f>IF($G61="","",IF($G61&lt;=0,"Out of stock",IF(AND($H61&lt;&gt;"",$G61&lt;=$H61),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="F62" s="3">
+        <f>IF($D62&gt;0,$E62/$D62,"")</f>
+        <v/>
+      </c>
+      <c r="G62" s="3">
+        <f>IF($D62="","",$D62-SUMIF(SKU_MATERIALS!$D:$D,$A62,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I62" s="3">
+        <f>IF($G62="","",IF($G62&lt;=0,"Out of stock",IF(AND($H62&lt;&gt;"",$G62&lt;=$H62),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="F63" s="3">
+        <f>IF($D63&gt;0,$E63/$D63,"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="3">
+        <f>IF($D63="","",$D63-SUMIF(SKU_MATERIALS!$D:$D,$A63,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I63" s="3">
+        <f>IF($G63="","",IF($G63&lt;=0,"Out of stock",IF(AND($H63&lt;&gt;"",$G63&lt;=$H63),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="F64" s="3">
+        <f>IF($D64&gt;0,$E64/$D64,"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="3">
+        <f>IF($D64="","",$D64-SUMIF(SKU_MATERIALS!$D:$D,$A64,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I64" s="3">
+        <f>IF($G64="","",IF($G64&lt;=0,"Out of stock",IF(AND($H64&lt;&gt;"",$G64&lt;=$H64),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="F65" s="3">
+        <f>IF($D65&gt;0,$E65/$D65,"")</f>
+        <v/>
+      </c>
+      <c r="G65" s="3">
+        <f>IF($D65="","",$D65-SUMIF(SKU_MATERIALS!$D:$D,$A65,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I65" s="3">
+        <f>IF($G65="","",IF($G65&lt;=0,"Out of stock",IF(AND($H65&lt;&gt;"",$G65&lt;=$H65),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="F66" s="3">
+        <f>IF($D66&gt;0,$E66/$D66,"")</f>
+        <v/>
+      </c>
+      <c r="G66" s="3">
+        <f>IF($D66="","",$D66-SUMIF(SKU_MATERIALS!$D:$D,$A66,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I66" s="3">
+        <f>IF($G66="","",IF($G66&lt;=0,"Out of stock",IF(AND($H66&lt;&gt;"",$G66&lt;=$H66),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="F67" s="3">
+        <f>IF($D67&gt;0,$E67/$D67,"")</f>
+        <v/>
+      </c>
+      <c r="G67" s="3">
+        <f>IF($D67="","",$D67-SUMIF(SKU_MATERIALS!$D:$D,$A67,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I67" s="3">
+        <f>IF($G67="","",IF($G67&lt;=0,"Out of stock",IF(AND($H67&lt;&gt;"",$G67&lt;=$H67),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="F68" s="3">
+        <f>IF($D68&gt;0,$E68/$D68,"")</f>
+        <v/>
+      </c>
+      <c r="G68" s="3">
+        <f>IF($D68="","",$D68-SUMIF(SKU_MATERIALS!$D:$D,$A68,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I68" s="3">
+        <f>IF($G68="","",IF($G68&lt;=0,"Out of stock",IF(AND($H68&lt;&gt;"",$G68&lt;=$H68),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="F69" s="3">
+        <f>IF($D69&gt;0,$E69/$D69,"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="3">
+        <f>IF($D69="","",$D69-SUMIF(SKU_MATERIALS!$D:$D,$A69,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I69" s="3">
+        <f>IF($G69="","",IF($G69&lt;=0,"Out of stock",IF(AND($H69&lt;&gt;"",$G69&lt;=$H69),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="F70" s="3">
+        <f>IF($D70&gt;0,$E70/$D70,"")</f>
+        <v/>
+      </c>
+      <c r="G70" s="3">
+        <f>IF($D70="","",$D70-SUMIF(SKU_MATERIALS!$D:$D,$A70,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I70" s="3">
+        <f>IF($G70="","",IF($G70&lt;=0,"Out of stock",IF(AND($H70&lt;&gt;"",$G70&lt;=$H70),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="F71" s="3">
+        <f>IF($D71&gt;0,$E71/$D71,"")</f>
+        <v/>
+      </c>
+      <c r="G71" s="3">
+        <f>IF($D71="","",$D71-SUMIF(SKU_MATERIALS!$D:$D,$A71,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I71" s="3">
+        <f>IF($G71="","",IF($G71&lt;=0,"Out of stock",IF(AND($H71&lt;&gt;"",$G71&lt;=$H71),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="F72" s="3">
+        <f>IF($D72&gt;0,$E72/$D72,"")</f>
+        <v/>
+      </c>
+      <c r="G72" s="3">
+        <f>IF($D72="","",$D72-SUMIF(SKU_MATERIALS!$D:$D,$A72,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I72" s="3">
+        <f>IF($G72="","",IF($G72&lt;=0,"Out of stock",IF(AND($H72&lt;&gt;"",$G72&lt;=$H72),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="F73" s="3">
+        <f>IF($D73&gt;0,$E73/$D73,"")</f>
+        <v/>
+      </c>
+      <c r="G73" s="3">
+        <f>IF($D73="","",$D73-SUMIF(SKU_MATERIALS!$D:$D,$A73,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I73" s="3">
+        <f>IF($G73="","",IF($G73&lt;=0,"Out of stock",IF(AND($H73&lt;&gt;"",$G73&lt;=$H73),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="F74" s="3">
+        <f>IF($D74&gt;0,$E74/$D74,"")</f>
+        <v/>
+      </c>
+      <c r="G74" s="3">
+        <f>IF($D74="","",$D74-SUMIF(SKU_MATERIALS!$D:$D,$A74,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I74" s="3">
+        <f>IF($G74="","",IF($G74&lt;=0,"Out of stock",IF(AND($H74&lt;&gt;"",$G74&lt;=$H74),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="F75" s="3">
+        <f>IF($D75&gt;0,$E75/$D75,"")</f>
+        <v/>
+      </c>
+      <c r="G75" s="3">
+        <f>IF($D75="","",$D75-SUMIF(SKU_MATERIALS!$D:$D,$A75,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I75" s="3">
+        <f>IF($G75="","",IF($G75&lt;=0,"Out of stock",IF(AND($H75&lt;&gt;"",$G75&lt;=$H75),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="F76" s="3">
+        <f>IF($D76&gt;0,$E76/$D76,"")</f>
+        <v/>
+      </c>
+      <c r="G76" s="3">
+        <f>IF($D76="","",$D76-SUMIF(SKU_MATERIALS!$D:$D,$A76,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I76" s="3">
+        <f>IF($G76="","",IF($G76&lt;=0,"Out of stock",IF(AND($H76&lt;&gt;"",$G76&lt;=$H76),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="F77" s="3">
+        <f>IF($D77&gt;0,$E77/$D77,"")</f>
+        <v/>
+      </c>
+      <c r="G77" s="3">
+        <f>IF($D77="","",$D77-SUMIF(SKU_MATERIALS!$D:$D,$A77,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I77" s="3">
+        <f>IF($G77="","",IF($G77&lt;=0,"Out of stock",IF(AND($H77&lt;&gt;"",$G77&lt;=$H77),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="F78" s="3">
+        <f>IF($D78&gt;0,$E78/$D78,"")</f>
+        <v/>
+      </c>
+      <c r="G78" s="3">
+        <f>IF($D78="","",$D78-SUMIF(SKU_MATERIALS!$D:$D,$A78,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I78" s="3">
+        <f>IF($G78="","",IF($G78&lt;=0,"Out of stock",IF(AND($H78&lt;&gt;"",$G78&lt;=$H78),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="F79" s="3">
+        <f>IF($D79&gt;0,$E79/$D79,"")</f>
+        <v/>
+      </c>
+      <c r="G79" s="3">
+        <f>IF($D79="","",$D79-SUMIF(SKU_MATERIALS!$D:$D,$A79,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I79" s="3">
+        <f>IF($G79="","",IF($G79&lt;=0,"Out of stock",IF(AND($H79&lt;&gt;"",$G79&lt;=$H79),"Running low","In stock")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="F80" s="3">
+        <f>IF($D80&gt;0,$E80/$D80,"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="3">
+        <f>IF($D80="","",$D80-SUMIF(SKU_MATERIALS!$D:$D,$A80,SKU_MATERIALS!$F:$F))</f>
+        <v/>
+      </c>
+      <c r="I80" s="3">
+        <f>IF($G80="","",IF($G80&lt;=0,"Out of stock",IF(AND($H80&lt;&gt;"",$G80&lt;=$H80),"Running low","In stock")))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Fabric,Thread,Paint,Dye,Button,Trim,Packaging,Article,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"metre,spool,jar,piece,packet,kg,set"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"In stock,Running low,Out of stock"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5658,114 +6757,1559 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>sku</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>style_family</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>material</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>use_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>qty_used</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>rate</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HB1HE-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bamboo fabric</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>metre</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>HB1HE-HH</t>
+        </is>
+      </c>
+      <c r="C2" s="3">
+        <f>IFERROR(VLOOKUP($B2,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Bamboo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3">
+        <f>IFERROR(VLOOKUP($D2,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H2" s="3">
+        <f>IFERROR(VLOOKUP($D2,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I2" s="3">
+        <f>IF(AND($F2&lt;&gt;"",$H2&lt;&gt;""),$F2*$H2,"")</f>
+        <v/>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>shirt body</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HB1HE-01</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Black thread</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>spool</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>embroidery</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>28/06/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="3">
+        <f>IFERROR(VLOOKUP($B3,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Bamboo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="3">
+        <f>IFERROR(VLOOKUP($D3,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H3" s="3">
+        <f>IFERROR(VLOOKUP($D3,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I3" s="3">
+        <f>IF(AND($F3&lt;&gt;"",$H3&lt;&gt;""),$F3*$H3,"")</f>
+        <v/>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>sampling</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HB1UHP-01</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Wooden buttons</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>piece</t>
-        </is>
+      <c r="C4" s="3">
+        <f>IFERROR(VLOOKUP($B4,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="3">
+        <f>IFERROR(VLOOKUP($D4,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H4" s="3">
+        <f>IFERROR(VLOOKUP($D4,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I4" s="3">
+        <f>IF(AND($F4&lt;&gt;"",$H4&lt;&gt;""),$F4*$H4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" s="3">
+        <f>IFERROR(VLOOKUP($B5,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="3">
+        <f>IFERROR(VLOOKUP($D5,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="3">
+        <f>IFERROR(VLOOKUP($D5,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I5" s="3">
+        <f>IF(AND($F5&lt;&gt;"",$H5&lt;&gt;""),$F5*$H5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="3">
+        <f>IFERROR(VLOOKUP($B6,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="3">
+        <f>IFERROR(VLOOKUP($D6,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="3">
+        <f>IFERROR(VLOOKUP($D6,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I6" s="3">
+        <f>IF(AND($F6&lt;&gt;"",$H6&lt;&gt;""),$F6*$H6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="3">
+        <f>IFERROR(VLOOKUP($B7,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="3">
+        <f>IFERROR(VLOOKUP($D7,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="3">
+        <f>IFERROR(VLOOKUP($D7,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="3">
+        <f>IF(AND($F7&lt;&gt;"",$H7&lt;&gt;""),$F7*$H7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="3">
+        <f>IFERROR(VLOOKUP($B8,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="3">
+        <f>IFERROR(VLOOKUP($D8,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="3">
+        <f>IFERROR(VLOOKUP($D8,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="3">
+        <f>IF(AND($F8&lt;&gt;"",$H8&lt;&gt;""),$F8*$H8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="3">
+        <f>IFERROR(VLOOKUP($B9,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>IFERROR(VLOOKUP($D9,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="3">
+        <f>IFERROR(VLOOKUP($D9,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="3">
+        <f>IF(AND($F9&lt;&gt;"",$H9&lt;&gt;""),$F9*$H9,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="3">
+        <f>IFERROR(VLOOKUP($B10,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="3">
+        <f>IFERROR(VLOOKUP($D10,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="3">
+        <f>IFERROR(VLOOKUP($D10,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="3">
+        <f>IF(AND($F10&lt;&gt;"",$H10&lt;&gt;""),$F10*$H10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="3">
+        <f>IFERROR(VLOOKUP($B11,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>IFERROR(VLOOKUP($D11,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="3">
+        <f>IFERROR(VLOOKUP($D11,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="3">
+        <f>IF(AND($F11&lt;&gt;"",$H11&lt;&gt;""),$F11*$H11,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="3">
+        <f>IFERROR(VLOOKUP($B12,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="3">
+        <f>IFERROR(VLOOKUP($D12,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="3">
+        <f>IFERROR(VLOOKUP($D12,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="3">
+        <f>IF(AND($F12&lt;&gt;"",$H12&lt;&gt;""),$F12*$H12,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="3">
+        <f>IFERROR(VLOOKUP($B13,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="3">
+        <f>IFERROR(VLOOKUP($D13,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="3">
+        <f>IFERROR(VLOOKUP($D13,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="3">
+        <f>IF(AND($F13&lt;&gt;"",$H13&lt;&gt;""),$F13*$H13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="3">
+        <f>IFERROR(VLOOKUP($B14,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="3">
+        <f>IFERROR(VLOOKUP($D14,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="3">
+        <f>IFERROR(VLOOKUP($D14,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="3">
+        <f>IF(AND($F14&lt;&gt;"",$H14&lt;&gt;""),$F14*$H14,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3">
+        <f>IFERROR(VLOOKUP($B15,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="3">
+        <f>IFERROR(VLOOKUP($D15,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="3">
+        <f>IFERROR(VLOOKUP($D15,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="3">
+        <f>IF(AND($F15&lt;&gt;"",$H15&lt;&gt;""),$F15*$H15,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="3">
+        <f>IFERROR(VLOOKUP($B16,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="3">
+        <f>IFERROR(VLOOKUP($D16,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="3">
+        <f>IFERROR(VLOOKUP($D16,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="3">
+        <f>IF(AND($F16&lt;&gt;"",$H16&lt;&gt;""),$F16*$H16,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="3">
+        <f>IFERROR(VLOOKUP($B17,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="3">
+        <f>IFERROR(VLOOKUP($D17,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="3">
+        <f>IFERROR(VLOOKUP($D17,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="3">
+        <f>IF(AND($F17&lt;&gt;"",$H17&lt;&gt;""),$F17*$H17,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="3">
+        <f>IFERROR(VLOOKUP($B18,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="3">
+        <f>IFERROR(VLOOKUP($D18,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="3">
+        <f>IFERROR(VLOOKUP($D18,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="3">
+        <f>IF(AND($F18&lt;&gt;"",$H18&lt;&gt;""),$F18*$H18,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="3">
+        <f>IFERROR(VLOOKUP($B19,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="3">
+        <f>IFERROR(VLOOKUP($D19,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="3">
+        <f>IFERROR(VLOOKUP($D19,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="3">
+        <f>IF(AND($F19&lt;&gt;"",$H19&lt;&gt;""),$F19*$H19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="3">
+        <f>IFERROR(VLOOKUP($B20,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="3">
+        <f>IFERROR(VLOOKUP($D20,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="3">
+        <f>IFERROR(VLOOKUP($D20,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="3">
+        <f>IF(AND($F20&lt;&gt;"",$H20&lt;&gt;""),$F20*$H20,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="3">
+        <f>IFERROR(VLOOKUP($B21,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="3">
+        <f>IFERROR(VLOOKUP($D21,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="3">
+        <f>IFERROR(VLOOKUP($D21,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="3">
+        <f>IF(AND($F21&lt;&gt;"",$H21&lt;&gt;""),$F21*$H21,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="3">
+        <f>IFERROR(VLOOKUP($B22,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="3">
+        <f>IFERROR(VLOOKUP($D22,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="3">
+        <f>IFERROR(VLOOKUP($D22,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="3">
+        <f>IF(AND($F22&lt;&gt;"",$H22&lt;&gt;""),$F22*$H22,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" s="3">
+        <f>IFERROR(VLOOKUP($B23,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="3">
+        <f>IFERROR(VLOOKUP($D23,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="3">
+        <f>IFERROR(VLOOKUP($D23,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="3">
+        <f>IF(AND($F23&lt;&gt;"",$H23&lt;&gt;""),$F23*$H23,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="3">
+        <f>IFERROR(VLOOKUP($B24,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="3">
+        <f>IFERROR(VLOOKUP($D24,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="3">
+        <f>IFERROR(VLOOKUP($D24,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="3">
+        <f>IF(AND($F24&lt;&gt;"",$H24&lt;&gt;""),$F24*$H24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="3">
+        <f>IFERROR(VLOOKUP($B25,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="3">
+        <f>IFERROR(VLOOKUP($D25,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="3">
+        <f>IFERROR(VLOOKUP($D25,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="3">
+        <f>IF(AND($F25&lt;&gt;"",$H25&lt;&gt;""),$F25*$H25,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" s="3">
+        <f>IFERROR(VLOOKUP($B26,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="3">
+        <f>IFERROR(VLOOKUP($D26,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="3">
+        <f>IFERROR(VLOOKUP($D26,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="3">
+        <f>IF(AND($F26&lt;&gt;"",$H26&lt;&gt;""),$F26*$H26,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" s="3">
+        <f>IFERROR(VLOOKUP($B27,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="3">
+        <f>IFERROR(VLOOKUP($D27,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="3">
+        <f>IFERROR(VLOOKUP($D27,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="3">
+        <f>IF(AND($F27&lt;&gt;"",$H27&lt;&gt;""),$F27*$H27,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" s="3">
+        <f>IFERROR(VLOOKUP($B28,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="3">
+        <f>IFERROR(VLOOKUP($D28,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="3">
+        <f>IFERROR(VLOOKUP($D28,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="3">
+        <f>IF(AND($F28&lt;&gt;"",$H28&lt;&gt;""),$F28*$H28,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="3">
+        <f>IFERROR(VLOOKUP($B29,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="3">
+        <f>IFERROR(VLOOKUP($D29,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H29" s="3">
+        <f>IFERROR(VLOOKUP($D29,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="3">
+        <f>IF(AND($F29&lt;&gt;"",$H29&lt;&gt;""),$F29*$H29,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" s="3">
+        <f>IFERROR(VLOOKUP($B30,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="3">
+        <f>IFERROR(VLOOKUP($D30,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H30" s="3">
+        <f>IFERROR(VLOOKUP($D30,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="3">
+        <f>IF(AND($F30&lt;&gt;"",$H30&lt;&gt;""),$F30*$H30,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="3">
+        <f>IFERROR(VLOOKUP($B31,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="3">
+        <f>IFERROR(VLOOKUP($D31,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H31" s="3">
+        <f>IFERROR(VLOOKUP($D31,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="3">
+        <f>IF(AND($F31&lt;&gt;"",$H31&lt;&gt;""),$F31*$H31,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="3">
+        <f>IFERROR(VLOOKUP($B32,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G32" s="3">
+        <f>IFERROR(VLOOKUP($D32,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H32" s="3">
+        <f>IFERROR(VLOOKUP($D32,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="3">
+        <f>IF(AND($F32&lt;&gt;"",$H32&lt;&gt;""),$F32*$H32,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="3">
+        <f>IFERROR(VLOOKUP($B33,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="3">
+        <f>IFERROR(VLOOKUP($D33,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H33" s="3">
+        <f>IFERROR(VLOOKUP($D33,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="3">
+        <f>IF(AND($F33&lt;&gt;"",$H33&lt;&gt;""),$F33*$H33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" s="3">
+        <f>IFERROR(VLOOKUP($B34,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="3">
+        <f>IFERROR(VLOOKUP($D34,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="3">
+        <f>IFERROR(VLOOKUP($D34,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="3">
+        <f>IF(AND($F34&lt;&gt;"",$H34&lt;&gt;""),$F34*$H34,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="3">
+        <f>IFERROR(VLOOKUP($B35,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="3">
+        <f>IFERROR(VLOOKUP($D35,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="3">
+        <f>IFERROR(VLOOKUP($D35,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="3">
+        <f>IF(AND($F35&lt;&gt;"",$H35&lt;&gt;""),$F35*$H35,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" s="3">
+        <f>IFERROR(VLOOKUP($B36,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="3">
+        <f>IFERROR(VLOOKUP($D36,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="3">
+        <f>IFERROR(VLOOKUP($D36,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="3">
+        <f>IF(AND($F36&lt;&gt;"",$H36&lt;&gt;""),$F36*$H36,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" s="3">
+        <f>IFERROR(VLOOKUP($B37,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="3">
+        <f>IFERROR(VLOOKUP($D37,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="3">
+        <f>IFERROR(VLOOKUP($D37,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="3">
+        <f>IF(AND($F37&lt;&gt;"",$H37&lt;&gt;""),$F37*$H37,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" s="3">
+        <f>IFERROR(VLOOKUP($B38,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="3">
+        <f>IFERROR(VLOOKUP($D38,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="3">
+        <f>IFERROR(VLOOKUP($D38,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="3">
+        <f>IF(AND($F38&lt;&gt;"",$H38&lt;&gt;""),$F38*$H38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="C39" s="3">
+        <f>IFERROR(VLOOKUP($B39,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="3">
+        <f>IFERROR(VLOOKUP($D39,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H39" s="3">
+        <f>IFERROR(VLOOKUP($D39,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="3">
+        <f>IF(AND($F39&lt;&gt;"",$H39&lt;&gt;""),$F39*$H39,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" s="3">
+        <f>IFERROR(VLOOKUP($B40,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="3">
+        <f>IFERROR(VLOOKUP($D40,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="3">
+        <f>IFERROR(VLOOKUP($D40,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="3">
+        <f>IF(AND($F40&lt;&gt;"",$H40&lt;&gt;""),$F40*$H40,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41" s="3">
+        <f>IFERROR(VLOOKUP($B41,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="3">
+        <f>IFERROR(VLOOKUP($D41,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H41" s="3">
+        <f>IFERROR(VLOOKUP($D41,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I41" s="3">
+        <f>IF(AND($F41&lt;&gt;"",$H41&lt;&gt;""),$F41*$H41,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="3">
+        <f>IFERROR(VLOOKUP($B42,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G42" s="3">
+        <f>IFERROR(VLOOKUP($D42,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H42" s="3">
+        <f>IFERROR(VLOOKUP($D42,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I42" s="3">
+        <f>IF(AND($F42&lt;&gt;"",$H42&lt;&gt;""),$F42*$H42,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="3">
+        <f>IFERROR(VLOOKUP($B43,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="3">
+        <f>IFERROR(VLOOKUP($D43,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H43" s="3">
+        <f>IFERROR(VLOOKUP($D43,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I43" s="3">
+        <f>IF(AND($F43&lt;&gt;"",$H43&lt;&gt;""),$F43*$H43,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="3">
+        <f>IFERROR(VLOOKUP($B44,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="3">
+        <f>IFERROR(VLOOKUP($D44,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H44" s="3">
+        <f>IFERROR(VLOOKUP($D44,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="3">
+        <f>IF(AND($F44&lt;&gt;"",$H44&lt;&gt;""),$F44*$H44,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" s="3">
+        <f>IFERROR(VLOOKUP($B45,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="3">
+        <f>IFERROR(VLOOKUP($D45,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H45" s="3">
+        <f>IFERROR(VLOOKUP($D45,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I45" s="3">
+        <f>IF(AND($F45&lt;&gt;"",$H45&lt;&gt;""),$F45*$H45,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" s="3">
+        <f>IFERROR(VLOOKUP($B46,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="3">
+        <f>IFERROR(VLOOKUP($D46,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H46" s="3">
+        <f>IFERROR(VLOOKUP($D46,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="3">
+        <f>IF(AND($F46&lt;&gt;"",$H46&lt;&gt;""),$F46*$H46,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="3">
+        <f>IFERROR(VLOOKUP($B47,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="3">
+        <f>IFERROR(VLOOKUP($D47,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H47" s="3">
+        <f>IFERROR(VLOOKUP($D47,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I47" s="3">
+        <f>IF(AND($F47&lt;&gt;"",$H47&lt;&gt;""),$F47*$H47,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="3">
+        <f>IFERROR(VLOOKUP($B48,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="3">
+        <f>IFERROR(VLOOKUP($D48,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H48" s="3">
+        <f>IFERROR(VLOOKUP($D48,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="3">
+        <f>IF(AND($F48&lt;&gt;"",$H48&lt;&gt;""),$F48*$H48,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="3">
+        <f>IFERROR(VLOOKUP($B49,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="3">
+        <f>IFERROR(VLOOKUP($D49,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H49" s="3">
+        <f>IFERROR(VLOOKUP($D49,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="3">
+        <f>IF(AND($F49&lt;&gt;"",$H49&lt;&gt;""),$F49*$H49,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="C50" s="3">
+        <f>IFERROR(VLOOKUP($B50,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="3">
+        <f>IFERROR(VLOOKUP($D50,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H50" s="3">
+        <f>IFERROR(VLOOKUP($D50,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I50" s="3">
+        <f>IF(AND($F50&lt;&gt;"",$H50&lt;&gt;""),$F50*$H50,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="C51" s="3">
+        <f>IFERROR(VLOOKUP($B51,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="3">
+        <f>IFERROR(VLOOKUP($D51,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="3">
+        <f>IFERROR(VLOOKUP($D51,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="3">
+        <f>IF(AND($F51&lt;&gt;"",$H51&lt;&gt;""),$F51*$H51,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="C52" s="3">
+        <f>IFERROR(VLOOKUP($B52,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="3">
+        <f>IFERROR(VLOOKUP($D52,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H52" s="3">
+        <f>IFERROR(VLOOKUP($D52,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I52" s="3">
+        <f>IF(AND($F52&lt;&gt;"",$H52&lt;&gt;""),$F52*$H52,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="C53" s="3">
+        <f>IFERROR(VLOOKUP($B53,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="3">
+        <f>IFERROR(VLOOKUP($D53,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H53" s="3">
+        <f>IFERROR(VLOOKUP($D53,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I53" s="3">
+        <f>IF(AND($F53&lt;&gt;"",$H53&lt;&gt;""),$F53*$H53,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" s="3">
+        <f>IFERROR(VLOOKUP($B54,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="3">
+        <f>IFERROR(VLOOKUP($D54,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H54" s="3">
+        <f>IFERROR(VLOOKUP($D54,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I54" s="3">
+        <f>IF(AND($F54&lt;&gt;"",$H54&lt;&gt;""),$F54*$H54,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="3">
+        <f>IFERROR(VLOOKUP($B55,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="3">
+        <f>IFERROR(VLOOKUP($D55,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H55" s="3">
+        <f>IFERROR(VLOOKUP($D55,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I55" s="3">
+        <f>IF(AND($F55&lt;&gt;"",$H55&lt;&gt;""),$F55*$H55,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" s="3">
+        <f>IFERROR(VLOOKUP($B56,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="3">
+        <f>IFERROR(VLOOKUP($D56,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H56" s="3">
+        <f>IFERROR(VLOOKUP($D56,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I56" s="3">
+        <f>IF(AND($F56&lt;&gt;"",$H56&lt;&gt;""),$F56*$H56,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" s="3">
+        <f>IFERROR(VLOOKUP($B57,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="3">
+        <f>IFERROR(VLOOKUP($D57,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H57" s="3">
+        <f>IFERROR(VLOOKUP($D57,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I57" s="3">
+        <f>IF(AND($F57&lt;&gt;"",$H57&lt;&gt;""),$F57*$H57,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" s="3">
+        <f>IFERROR(VLOOKUP($B58,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="3">
+        <f>IFERROR(VLOOKUP($D58,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H58" s="3">
+        <f>IFERROR(VLOOKUP($D58,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I58" s="3">
+        <f>IF(AND($F58&lt;&gt;"",$H58&lt;&gt;""),$F58*$H58,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" s="3">
+        <f>IFERROR(VLOOKUP($B59,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="3">
+        <f>IFERROR(VLOOKUP($D59,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H59" s="3">
+        <f>IFERROR(VLOOKUP($D59,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I59" s="3">
+        <f>IF(AND($F59&lt;&gt;"",$H59&lt;&gt;""),$F59*$H59,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" s="3">
+        <f>IFERROR(VLOOKUP($B60,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="3">
+        <f>IFERROR(VLOOKUP($D60,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H60" s="3">
+        <f>IFERROR(VLOOKUP($D60,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I60" s="3">
+        <f>IF(AND($F60&lt;&gt;"",$H60&lt;&gt;""),$F60*$H60,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" s="3">
+        <f>IFERROR(VLOOKUP($B61,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="3">
+        <f>IFERROR(VLOOKUP($D61,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H61" s="3">
+        <f>IFERROR(VLOOKUP($D61,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="3">
+        <f>IF(AND($F61&lt;&gt;"",$H61&lt;&gt;""),$F61*$H61,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" s="3">
+        <f>IFERROR(VLOOKUP($B62,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G62" s="3">
+        <f>IFERROR(VLOOKUP($D62,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H62" s="3">
+        <f>IFERROR(VLOOKUP($D62,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I62" s="3">
+        <f>IF(AND($F62&lt;&gt;"",$H62&lt;&gt;""),$F62*$H62,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" s="3">
+        <f>IFERROR(VLOOKUP($B63,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="3">
+        <f>IFERROR(VLOOKUP($D63,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H63" s="3">
+        <f>IFERROR(VLOOKUP($D63,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I63" s="3">
+        <f>IF(AND($F63&lt;&gt;"",$H63&lt;&gt;""),$F63*$H63,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" s="3">
+        <f>IFERROR(VLOOKUP($B64,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="3">
+        <f>IFERROR(VLOOKUP($D64,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H64" s="3">
+        <f>IFERROR(VLOOKUP($D64,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I64" s="3">
+        <f>IF(AND($F64&lt;&gt;"",$H64&lt;&gt;""),$F64*$H64,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="C65" s="3">
+        <f>IFERROR(VLOOKUP($B65,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G65" s="3">
+        <f>IFERROR(VLOOKUP($D65,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H65" s="3">
+        <f>IFERROR(VLOOKUP($D65,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I65" s="3">
+        <f>IF(AND($F65&lt;&gt;"",$H65&lt;&gt;""),$F65*$H65,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" s="3">
+        <f>IFERROR(VLOOKUP($B66,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G66" s="3">
+        <f>IFERROR(VLOOKUP($D66,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H66" s="3">
+        <f>IFERROR(VLOOKUP($D66,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I66" s="3">
+        <f>IF(AND($F66&lt;&gt;"",$H66&lt;&gt;""),$F66*$H66,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" s="3">
+        <f>IFERROR(VLOOKUP($B67,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G67" s="3">
+        <f>IFERROR(VLOOKUP($D67,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H67" s="3">
+        <f>IFERROR(VLOOKUP($D67,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I67" s="3">
+        <f>IF(AND($F67&lt;&gt;"",$H67&lt;&gt;""),$F67*$H67,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" s="3">
+        <f>IFERROR(VLOOKUP($B68,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G68" s="3">
+        <f>IFERROR(VLOOKUP($D68,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H68" s="3">
+        <f>IFERROR(VLOOKUP($D68,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I68" s="3">
+        <f>IF(AND($F68&lt;&gt;"",$H68&lt;&gt;""),$F68*$H68,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" s="3">
+        <f>IFERROR(VLOOKUP($B69,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="3">
+        <f>IFERROR(VLOOKUP($D69,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H69" s="3">
+        <f>IFERROR(VLOOKUP($D69,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I69" s="3">
+        <f>IF(AND($F69&lt;&gt;"",$H69&lt;&gt;""),$F69*$H69,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" s="3">
+        <f>IFERROR(VLOOKUP($B70,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G70" s="3">
+        <f>IFERROR(VLOOKUP($D70,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H70" s="3">
+        <f>IFERROR(VLOOKUP($D70,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I70" s="3">
+        <f>IF(AND($F70&lt;&gt;"",$H70&lt;&gt;""),$F70*$H70,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" s="3">
+        <f>IFERROR(VLOOKUP($B71,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G71" s="3">
+        <f>IFERROR(VLOOKUP($D71,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H71" s="3">
+        <f>IFERROR(VLOOKUP($D71,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I71" s="3">
+        <f>IF(AND($F71&lt;&gt;"",$H71&lt;&gt;""),$F71*$H71,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" s="3">
+        <f>IFERROR(VLOOKUP($B72,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G72" s="3">
+        <f>IFERROR(VLOOKUP($D72,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H72" s="3">
+        <f>IFERROR(VLOOKUP($D72,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I72" s="3">
+        <f>IF(AND($F72&lt;&gt;"",$H72&lt;&gt;""),$F72*$H72,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" s="3">
+        <f>IFERROR(VLOOKUP($B73,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G73" s="3">
+        <f>IFERROR(VLOOKUP($D73,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H73" s="3">
+        <f>IFERROR(VLOOKUP($D73,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I73" s="3">
+        <f>IF(AND($F73&lt;&gt;"",$H73&lt;&gt;""),$F73*$H73,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="C74" s="3">
+        <f>IFERROR(VLOOKUP($B74,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G74" s="3">
+        <f>IFERROR(VLOOKUP($D74,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H74" s="3">
+        <f>IFERROR(VLOOKUP($D74,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I74" s="3">
+        <f>IF(AND($F74&lt;&gt;"",$H74&lt;&gt;""),$F74*$H74,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="C75" s="3">
+        <f>IFERROR(VLOOKUP($B75,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G75" s="3">
+        <f>IFERROR(VLOOKUP($D75,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H75" s="3">
+        <f>IFERROR(VLOOKUP($D75,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I75" s="3">
+        <f>IF(AND($F75&lt;&gt;"",$H75&lt;&gt;""),$F75*$H75,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="C76" s="3">
+        <f>IFERROR(VLOOKUP($B76,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G76" s="3">
+        <f>IFERROR(VLOOKUP($D76,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H76" s="3">
+        <f>IFERROR(VLOOKUP($D76,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I76" s="3">
+        <f>IF(AND($F76&lt;&gt;"",$H76&lt;&gt;""),$F76*$H76,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="C77" s="3">
+        <f>IFERROR(VLOOKUP($B77,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G77" s="3">
+        <f>IFERROR(VLOOKUP($D77,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H77" s="3">
+        <f>IFERROR(VLOOKUP($D77,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I77" s="3">
+        <f>IF(AND($F77&lt;&gt;"",$H77&lt;&gt;""),$F77*$H77,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="C78" s="3">
+        <f>IFERROR(VLOOKUP($B78,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G78" s="3">
+        <f>IFERROR(VLOOKUP($D78,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H78" s="3">
+        <f>IFERROR(VLOOKUP($D78,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I78" s="3">
+        <f>IF(AND($F78&lt;&gt;"",$H78&lt;&gt;""),$F78*$H78,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="C79" s="3">
+        <f>IFERROR(VLOOKUP($B79,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G79" s="3">
+        <f>IFERROR(VLOOKUP($D79,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H79" s="3">
+        <f>IFERROR(VLOOKUP($D79,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I79" s="3">
+        <f>IF(AND($F79&lt;&gt;"",$H79&lt;&gt;""),$F79*$H79,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="C80" s="3">
+        <f>IFERROR(VLOOKUP($B80,INVENTORY!$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="3">
+        <f>IFERROR(VLOOKUP($D80,MATERIALS!$A:$C,3,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="H80" s="3">
+        <f>IFERROR(VLOOKUP($D80,MATERIALS!$A:$F,6,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I80" s="3">
+        <f>IF(AND($F80&lt;&gt;"",$H80&lt;&gt;""),$F80*$H80,"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>INVENTORY!$A$2:$A$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>MATERIALS!$A$2:$A$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"R&amp;D,Production"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>